<commit_message>
chore: update stufe-5/dok/migrate-ig-to-ig-publisher-ptdata-1969 pages
</commit_message>
<xml_diff>
--- a/stufe-5/dok/migrate-ig-to-ig-publisher-ptdata-1969/all-profiles.xlsx
+++ b/stufe-5/dok/migrate-ig-to-ig-publisher-ptdata-1969/all-profiles.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5507" uniqueCount="657">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5705" uniqueCount="662">
   <si>
     <t>Property</t>
   </si>
@@ -2124,6 +2124,21 @@
   </si>
   <si>
     <t>May be identifiers or resources that caused the DocumentReference or referenced Document to be created.</t>
+  </si>
+  <si>
+    <t>ISiKTerminPriorityExtension</t>
+  </si>
+  <si>
+    <t>https://gematik.de/fhir/isik/StructureDefinition/ISiKTerminPriorityExtension</t>
+  </si>
+  <si>
+    <t>Diese Extension ermöglicht die strukturierte Angabe der Dringlichkeit (Priorität) eines Termins. Dies ist wichtig, um Notfälle oder besonders dringliche Termine im Buchungs- und Verwaltungssystem deutlich zu kennzeichnen und eine priorisierte Bearbeitung zu ermöglichen.</t>
+  </si>
+  <si>
+    <t>element:Appointment.priority</t>
+  </si>
+  <si>
+    <t>https://gematik.de/fhir/isik/ValueSet/ISiKTerminPriority</t>
   </si>
 </sst>
 </file>
@@ -2257,7 +2272,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B61"/>
+  <dimension ref="A1:B82"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="15.703125" customWidth="true"/>
@@ -2734,6 +2749,166 @@
         <v>34</v>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="B62" t="s" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s" s="2">
+        <v>2</v>
+      </c>
+      <c r="B63" t="s" s="2">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s" s="2">
+        <v>4</v>
+      </c>
+      <c r="B64" t="s" s="2">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s" s="2">
+        <v>6</v>
+      </c>
+      <c r="B65" t="s" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s" s="2">
+        <v>8</v>
+      </c>
+      <c r="B66" t="s" s="2">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s" s="2">
+        <v>9</v>
+      </c>
+      <c r="B67" s="2"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="s" s="2">
+        <v>11</v>
+      </c>
+      <c r="B68" t="s" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="B69" t="s" s="2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s" s="2">
+        <v>15</v>
+      </c>
+      <c r="B70" t="s" s="2">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="s" s="2">
+        <v>17</v>
+      </c>
+      <c r="B71" s="2"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="B72" t="s" s="2">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="B73" t="s" s="2">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="B74" s="2"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="s" s="2">
+        <v>23</v>
+      </c>
+      <c r="B75" s="2"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="s" s="2">
+        <v>24</v>
+      </c>
+      <c r="B76" t="s" s="2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="s" s="2">
+        <v>26</v>
+      </c>
+      <c r="B77" t="s" s="2">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="s" s="2">
+        <v>28</v>
+      </c>
+      <c r="B78" t="s" s="2">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="s" s="2">
+        <v>30</v>
+      </c>
+      <c r="B79" t="s" s="2">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="s" s="2">
+        <v>32</v>
+      </c>
+      <c r="B80" t="s" s="2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="B81" t="s" s="2">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="B82" t="s" s="2">
+        <v>660</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
@@ -2741,7 +2916,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AK162"/>
+  <dimension ref="A1:AK167"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="43.0625" customWidth="true" bestFit="true"/>
@@ -19817,6 +19992,521 @@
         <v>106</v>
       </c>
     </row>
+    <row r="163">
+      <c r="A163" t="s" s="2">
+        <v>657</v>
+      </c>
+      <c r="B163" t="s" s="2">
+        <v>29</v>
+      </c>
+      <c r="C163" t="s" s="2">
+        <v>29</v>
+      </c>
+      <c r="D163" s="2"/>
+      <c r="E163" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="F163" s="2"/>
+      <c r="G163" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="H163" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="I163" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="J163" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="K163" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="L163" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="M163" t="s" s="2">
+        <v>29</v>
+      </c>
+      <c r="N163" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="O163" s="2"/>
+      <c r="P163" s="2"/>
+      <c r="Q163" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="R163" s="2"/>
+      <c r="S163" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="T163" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="U163" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="V163" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="W163" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="X163" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="Y163" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="Z163" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AA163" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AB163" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AC163" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AD163" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AE163" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AF163" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AG163" t="s" s="2">
+        <v>29</v>
+      </c>
+      <c r="AH163" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AI163" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AJ163" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AK163" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="s" s="2">
+        <v>657</v>
+      </c>
+      <c r="B164" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="C164" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="D164" s="2"/>
+      <c r="E164" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="F164" s="2"/>
+      <c r="G164" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="H164" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="I164" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="J164" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="K164" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="L164" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="M164" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="N164" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="O164" s="2"/>
+      <c r="P164" s="2"/>
+      <c r="Q164" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="R164" s="2"/>
+      <c r="S164" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="T164" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="U164" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="V164" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="W164" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="X164" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="Y164" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="Z164" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AA164" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AB164" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AC164" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AD164" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AE164" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AF164" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AG164" t="s" s="2">
+        <v>86</v>
+      </c>
+      <c r="AH164" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AI164" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ164" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AK164" t="s" s="2">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="s" s="2">
+        <v>657</v>
+      </c>
+      <c r="B165" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="C165" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="D165" s="2"/>
+      <c r="E165" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="F165" s="2"/>
+      <c r="G165" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="H165" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I165" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="J165" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="K165" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="L165" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="M165" t="s" s="2">
+        <v>29</v>
+      </c>
+      <c r="N165" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="O165" s="2"/>
+      <c r="P165" s="2"/>
+      <c r="Q165" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="R165" s="2"/>
+      <c r="S165" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="T165" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="U165" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="V165" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="W165" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="X165" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="Y165" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="Z165" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AA165" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AB165" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AC165" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AD165" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="AE165" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AF165" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="AG165" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="AH165" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AI165" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AJ165" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AK165" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="s" s="2">
+        <v>657</v>
+      </c>
+      <c r="B166" t="s" s="2">
+        <v>94</v>
+      </c>
+      <c r="C166" t="s" s="2">
+        <v>94</v>
+      </c>
+      <c r="D166" s="2"/>
+      <c r="E166" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="F166" s="2"/>
+      <c r="G166" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="H166" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="I166" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="J166" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="K166" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="L166" t="s" s="2">
+        <v>95</v>
+      </c>
+      <c r="M166" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="N166" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="O166" t="s" s="2">
+        <v>98</v>
+      </c>
+      <c r="P166" s="2"/>
+      <c r="Q166" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="R166" s="2"/>
+      <c r="S166" t="s" s="2">
+        <v>658</v>
+      </c>
+      <c r="T166" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="U166" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="V166" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="W166" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="X166" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="Y166" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="Z166" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AA166" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AB166" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AC166" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AD166" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AE166" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AF166" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AG166" t="s" s="2">
+        <v>94</v>
+      </c>
+      <c r="AH166" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI166" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ166" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AK166" t="s" s="2">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="s" s="2">
+        <v>657</v>
+      </c>
+      <c r="B167" t="s" s="2">
+        <v>99</v>
+      </c>
+      <c r="C167" t="s" s="2">
+        <v>99</v>
+      </c>
+      <c r="D167" s="2"/>
+      <c r="E167" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="F167" s="2"/>
+      <c r="G167" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="H167" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="I167" t="s" s="2">
+        <v>117</v>
+      </c>
+      <c r="J167" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="K167" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="L167" t="s" s="2">
+        <v>263</v>
+      </c>
+      <c r="M167" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="N167" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="O167" s="2"/>
+      <c r="P167" s="2"/>
+      <c r="Q167" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="R167" s="2"/>
+      <c r="S167" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="T167" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="U167" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="V167" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="W167" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="X167" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="Y167" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="Z167" s="2"/>
+      <c r="AA167" t="s" s="2">
+        <v>661</v>
+      </c>
+      <c r="AB167" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AC167" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AD167" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AE167" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AF167" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AG167" t="s" s="2">
+        <v>99</v>
+      </c>
+      <c r="AH167" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AI167" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ167" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="AK167" t="s" s="2">
+        <v>106</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>